<commit_message>
refactor: restructure framework and improve code dynamism
</commit_message>
<xml_diff>
--- a/testdata/caldata.xlsx
+++ b/testdata/caldata.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="38">
   <si>
     <t>Principle</t>
   </si>
@@ -889,7 +889,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -941,6 +941,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="41" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="true"/>
@@ -1516,7 +1521,7 @@
       <c r="E2" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s" s="23">
+      <c r="F2" t="s" s="28">
         <v>14</v>
       </c>
     </row>
@@ -1536,7 +1541,7 @@
       <c r="E3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s" s="24">
+      <c r="F3" t="s" s="29">
         <v>14</v>
       </c>
     </row>
@@ -1556,7 +1561,7 @@
       <c r="E4" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F4" t="s" s="25">
+      <c r="F4" t="s" s="30">
         <v>14</v>
       </c>
     </row>
@@ -1576,7 +1581,7 @@
       <c r="E5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F5" t="s" s="26">
+      <c r="F5" t="s" s="31">
         <v>14</v>
       </c>
     </row>
@@ -1596,7 +1601,7 @@
       <c r="E6" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F6" t="s" s="27">
+      <c r="F6" t="s" s="32">
         <v>26</v>
       </c>
     </row>

</xml_diff>